<commit_message>
Module 2 initial commit
</commit_message>
<xml_diff>
--- a/data/results/stats_output.xlsx
+++ b/data/results/stats_output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/33119cfcffe101ac/Documents/Thesis/Thesis folder/conversational-group-rec-eval/data/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_CAF357543307005FF7286FC945B6AA6291AE5588" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E089926-4D83-44EA-ABDC-0CF58E556188}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="11_CAF357543307005FF7286FC945B6AA6291AE5588" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47608D9A-5365-4B8C-855A-BDA461968031}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1368" yWindow="1944" windowWidth="17280" windowHeight="9960" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consensus" sheetId="1" r:id="rId1"/>
@@ -583,6 +583,10 @@
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -795,6 +799,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
@@ -971,6 +978,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="4" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -1097,6 +1109,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="25.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">

</xml_diff>